<commit_message>
Correct Nachman Cohen invoice findings
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vhYGPaAM74nnJetAhxgmr
</commit_message>
<xml_diff>
--- a/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
+++ b/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
@@ -45,7 +45,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -55,7 +55,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -519,15 +519,19 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>לא נמצא</t>
+          <t>נמצא (כנראה, לפי שתי חשבוניות שהועלו)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>אין בתיבת המשרד אף מייל מנחמן אחרי אוגוסט 2025. החשבוניות האחרונות שהתקבלו הן 200388 (04/08/26) ו-200384 (03/06/26), ושתיהן ב-2,280 ₪ ולא ב-1,180 ₪ (נקראו מהדרייב).</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr"/>
+          <t>חשבונית 200389 (03/09/26, שירות אוגוסט 2026) וחשבונית 200391 (08/10/26, שירות ספטמבר 2026): כל אחת 1,000 ₪ + מע"מ 18% = 1,180 ₪. הן מתאימות לשתי ההעברות של 1,180 ₪ מ-13/10. החשבוניות הועלו ישירות לשיחה, וההתאמה לתאריכים של ההעברות לא נבדקה מול הבנק.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>קבצים: OADS-Invoice-200389.PDF, OADS-Invoice-200391.PDF</t>
+        </is>
+      </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>לא (אין שליחה לביזיבוקס אחרי 07/09/26)</t>
@@ -555,13 +559,13 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>אין חשבונית של 1,180 ₪. 200388 היא 2,280 ₪ (שירות יולי 2026, הופקה 04/08). ייתכן שההעברות של 1,180 ₪ הן תשלום חלקי על חשבונית של 2,280 ₪.</t>
+          <t>לא נמצאה חשבונית שמתאימה להעברה הזו. כנראה זו חשבונית של חודש יוני. בדרייב יש 200384 (03/06/26, שירות מאי) ו-200388 (04/08/26, שירות יולי), אבל הסכומים שלהן לא אומתו כי טקסט ה-PDF בדרייב לא אמין.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr"/>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>200388 נשלחה בחלק 1-5 של יולי-אוגוסט (07/09/26). חשבונית ב-1,180 ₪ לא נשלחה</t>
+          <t>200388 נשלחה בחלק 1-5 של יולי-אוגוסט (07/09/26)</t>
         </is>
       </c>
     </row>
@@ -579,7 +583,7 @@
       <c r="C4" s="2" t="n">
         <v>3983</v>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -610,7 +614,7 @@
       <c r="C5" s="2" t="n">
         <v>4142</v>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -645,7 +649,7 @@
       <c r="C6" s="2" t="n">
         <v>385</v>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -676,7 +680,7 @@
       <c r="C7" s="2" t="n">
         <v>375</v>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -742,7 +746,7 @@
       <c r="C9" s="2" t="n">
         <v>608</v>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>נמצא (סביר, הסכום לא אומת)</t>
         </is>
@@ -777,7 +781,7 @@
       <c r="C10" s="2" t="n">
         <v>350</v>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>נמצא (בתיבה)</t>
         </is>
@@ -812,7 +816,7 @@
       <c r="C11" s="2" t="n">
         <v>150</v>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -843,7 +847,7 @@
       <c r="C12" s="2" t="n">
         <v>130</v>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -874,7 +878,7 @@
       <c r="C13" s="2" t="n">
         <v>130</v>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -905,7 +909,7 @@
       <c r="C14" s="2" t="n">
         <v>1537</v>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -936,7 +940,7 @@
       <c r="C15" s="2" t="n">
         <v>298.32</v>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -967,7 +971,7 @@
       <c r="C16" s="2" t="n">
         <v>31.88</v>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -998,7 +1002,7 @@
       <c r="C17" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1029,7 +1033,7 @@
       <c r="C18" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1060,7 +1064,7 @@
       <c r="C19" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1091,7 +1095,7 @@
       <c r="C20" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1227,7 +1231,7 @@
       <c r="C24" s="2" t="n">
         <v>8322</v>
       </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1282,7 +1286,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>חשבוניות על שלוש העברות של 1,180 ₪ (15/07, 13/10 x2) והסבר: חשבוניות 200384 ו-200388 הן 2,280 ₪ כל אחת. האם 1,180 ₪ הוא תשלום חלקי?</t>
+          <t>חשבונית על העברת 1,180 ₪ מ-15/07 (כנראה שירות יוני). שתי ההעברות מ-13/10 כנראה מכוסות בחשבוניות 200389 ו-200391</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Nachman Cohen 15/07 covered by invoice 200385
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vhYGPaAM74nnJetAhxgmr
</commit_message>
<xml_diff>
--- a/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
+++ b/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
@@ -50,12 +50,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -552,20 +552,24 @@
       <c r="C3" s="2" t="n">
         <v>1180</v>
       </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>לא נמצא (לבדוק)</t>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>נמצא (חשבונית הועלתה לשיחה)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>לא נמצאה חשבונית שמתאימה להעברה הזו. כל חשבוניות נחמן הן 1,180 ₪. בדרייב יש 200384 (03/06/26, שירות מאי, כנראה מכוסה בהעברה מ-24/06) ו-200388 (04/08/26, שירות יולי). חשבונית של חודש יוני (שהופקה בתחילת יולי) לא נמצאה.</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr"/>
+          <t>חשבונית 200385 (07/07/26, שירות יוני 2026): 1,000 ₪ + מע"מ 18% = 1,180 ₪. מתאימה להעברה מ-15/07. ההתאמה לבנק לא נבדקה.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>קובץ: OADS-Invoice-200385.PDF</t>
+        </is>
+      </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>200388 נשלחה בחלק 1-5 של יולי-אוגוסט (07/09/26)</t>
+          <t>לא ידוע. 200385 לא הופיעה ברשימת הקבצים שנשלחו ביולי-אוגוסט (07/09/26), ולכן כנראה לא נשלחה</t>
         </is>
       </c>
     </row>
@@ -583,7 +587,7 @@
       <c r="C4" s="2" t="n">
         <v>3983</v>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -614,7 +618,7 @@
       <c r="C5" s="2" t="n">
         <v>4142</v>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -649,7 +653,7 @@
       <c r="C6" s="2" t="n">
         <v>385</v>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -680,7 +684,7 @@
       <c r="C7" s="2" t="n">
         <v>375</v>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -711,7 +715,7 @@
       <c r="C8" s="2" t="n">
         <v>296</v>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>נמצא קשור (לבדוק)</t>
         </is>
@@ -816,7 +820,7 @@
       <c r="C11" s="2" t="n">
         <v>150</v>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -847,7 +851,7 @@
       <c r="C12" s="2" t="n">
         <v>130</v>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -878,7 +882,7 @@
       <c r="C13" s="2" t="n">
         <v>130</v>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -909,7 +913,7 @@
       <c r="C14" s="2" t="n">
         <v>1537</v>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -940,7 +944,7 @@
       <c r="C15" s="2" t="n">
         <v>298.32</v>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -971,7 +975,7 @@
       <c r="C16" s="2" t="n">
         <v>31.88</v>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1002,7 +1006,7 @@
       <c r="C17" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1033,7 +1037,7 @@
       <c r="C18" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1064,7 +1068,7 @@
       <c r="C19" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1095,7 +1099,7 @@
       <c r="C20" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1126,7 +1130,7 @@
       <c r="C21" s="2" t="n">
         <v>878</v>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>נמצא חלקי (פוליסה)</t>
         </is>
@@ -1161,7 +1165,7 @@
       <c r="C22" s="2" t="n">
         <v>2179.25</v>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>נמצא חלקי (פוליסה)</t>
         </is>
@@ -1196,7 +1200,7 @@
       <c r="C23" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>נמצא חלקי (בעמלות לבדוק)</t>
         </is>
@@ -1231,7 +1235,7 @@
       <c r="C24" s="2" t="n">
         <v>8322</v>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1286,7 +1290,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>חשבונית על העברת 1,180 ₪ מ-15/07 (כנראה שירות יוני). שתי ההעברות מ-13/10 כנראה מכוסות בחשבוניות 200389 ו-200391</t>
+          <t>כל ההעברות של נחמן כהן מכוסות (200385, 200389, 200391). נשאר רק לשלוח אותן לביזיבוקס</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mika receipts 3067 and 3084
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vhYGPaAM74nnJetAhxgmr
</commit_message>
<xml_diff>
--- a/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
+++ b/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
@@ -50,12 +50,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -589,18 +589,22 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>לא נמצא</t>
+          <t>לא נמצא (לבדוק)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>אין חשבונית בסכום הזה. הכי קרוב: 3076 (4,525 ₪, 06/08/26) ו-3079 (4,339 ₪, 10/09/26), שתיהן בדרייב.</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr"/>
+          <t>חשבונית מס קבלה 3067 שהועלתה היא 3,981 ₪, מ-17/06/26, על חשבון עסקה 7057 (שירותי משרד מאי), ושולמה בהעברה ב-17/06. היא לא תואמת: הסכום שונה ב-2 ₪, והתאריך הוא 17/06 ולא 15/07. נמצאו עוד 3076 (4,525 ₪, 06/08/26) ו-3079 (4,339 ₪, 10/09/26).</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>קובץ: InvoiceReceipt_3067.pdf</t>
+        </is>
+      </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>3076 נשלחה (07/09/26). 3079 לא נשלחה</t>
+          <t>3067: כנראה נשלחה בדוחות מאי-יוני (לא נבדק). 3076 נשלחה (07/09/26). 3079 לא נשלחה</t>
         </is>
       </c>
     </row>
@@ -618,24 +622,24 @@
       <c r="C5" s="2" t="n">
         <v>4142</v>
       </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>לא נמצא</t>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>נמצא (חשבונית הועלתה לשיחה)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>נמצא רק חשבון עסקה 7079 מ-11/10/26 (invoice4u). חשבונית מס קבלה לא התקבלה.</t>
+          <t>חשבונית מס קבלה 3084 מ-14/10/26: 4,142 ₪ (3,509.80 + מע"מ 18%, 631.76 + עיגול 0.44). על חשבון עסקה 7079 (שירותי משרד ספטמבר), ושולמה בהעברה בנקאית ב-13/10/26.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>הודעה: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1878755242651072125</t>
+          <t>קובץ: InvoiceReceipt_3084.pdf</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>לא (חשבון עסקה אינו מסמך מס)</t>
+          <t>לא (אחרי 07/09/26)</t>
         </is>
       </c>
     </row>
@@ -653,7 +657,7 @@
       <c r="C6" s="2" t="n">
         <v>385</v>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -684,7 +688,7 @@
       <c r="C7" s="2" t="n">
         <v>375</v>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -715,7 +719,7 @@
       <c r="C8" s="2" t="n">
         <v>296</v>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>נמצא קשור (לבדוק)</t>
         </is>
@@ -820,7 +824,7 @@
       <c r="C11" s="2" t="n">
         <v>150</v>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -851,7 +855,7 @@
       <c r="C12" s="2" t="n">
         <v>130</v>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -882,7 +886,7 @@
       <c r="C13" s="2" t="n">
         <v>130</v>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -913,7 +917,7 @@
       <c r="C14" s="2" t="n">
         <v>1537</v>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -944,7 +948,7 @@
       <c r="C15" s="2" t="n">
         <v>298.32</v>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -975,7 +979,7 @@
       <c r="C16" s="2" t="n">
         <v>31.88</v>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1006,7 +1010,7 @@
       <c r="C17" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1037,7 +1041,7 @@
       <c r="C18" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1068,7 +1072,7 @@
       <c r="C19" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1099,7 +1103,7 @@
       <c r="C20" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1130,7 +1134,7 @@
       <c r="C21" s="2" t="n">
         <v>878</v>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>נמצא חלקי (פוליסה)</t>
         </is>
@@ -1165,7 +1169,7 @@
       <c r="C22" s="2" t="n">
         <v>2179.25</v>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>נמצא חלקי (פוליסה)</t>
         </is>
@@ -1200,7 +1204,7 @@
       <c r="C23" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>נמצא חלקי (בעמלות לבדוק)</t>
         </is>
@@ -1235,7 +1239,7 @@
       <c r="C24" s="2" t="n">
         <v>8322</v>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1302,7 +1306,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>חשבונית מס קבלה על 3,983 ₪ (15/07) ועל 4,142 ₪ (13/10, מקביל לחשבון עסקה 7079)</t>
+          <t>חשבונית מס קבלה על העברה של 3,983 ₪ מ-15/07 (4,142 ₪ מ-13/10 כבר סגורה בחשבונית 3084)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mika 3,983 matched to receipt 3067
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vhYGPaAM74nnJetAhxgmr
</commit_message>
<xml_diff>
--- a/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
+++ b/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
@@ -50,12 +50,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -587,14 +587,14 @@
       <c r="C4" s="2" t="n">
         <v>3983</v>
       </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>לא נמצא (לבדוק)</t>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>נמצא (חשבונית הועלתה לשיחה, פער של 2 ₪)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>חשבונית מס קבלה 3067 שהועלתה היא 3,981 ₪, מ-17/06/26, על חשבון עסקה 7057 (שירותי משרד מאי), ושולמה בהעברה ב-17/06. היא לא תואמת: הסכום שונה ב-2 ₪, והתאריך הוא 17/06 ולא 15/07. נמצאו עוד 3076 (4,525 ₪, 06/08/26) ו-3079 (4,339 ₪, 10/09/26).</t>
+          <t>חשבונית מס קבלה 3067 מ-17/06/26: 3,981 ₪, על חשבון עסקה 7057 (שירותי משרד מאי). בבנק רשומים 3,983 ₪, כלומר פער של 2 ₪. לפי ההנחיה, זו החשבונית המתאימה והפער הוא טעות. בקבלה עצמה רשום תשלום בהעברה ב-17/06 ולא ב-15/07.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -604,7 +604,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>3067: כנראה נשלחה בדוחות מאי-יוני (לא נבדק). 3076 נשלחה (07/09/26). 3079 לא נשלחה</t>
+          <t>לא ידוע. 3067 הופיעה בדרייב ב-21/06, ולא נבדק אם נשלחה</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       <c r="C6" s="2" t="n">
         <v>385</v>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -688,7 +688,7 @@
       <c r="C7" s="2" t="n">
         <v>375</v>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -719,7 +719,7 @@
       <c r="C8" s="2" t="n">
         <v>296</v>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>נמצא קשור (לבדוק)</t>
         </is>
@@ -824,7 +824,7 @@
       <c r="C11" s="2" t="n">
         <v>150</v>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -855,7 +855,7 @@
       <c r="C12" s="2" t="n">
         <v>130</v>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -886,7 +886,7 @@
       <c r="C13" s="2" t="n">
         <v>130</v>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -917,7 +917,7 @@
       <c r="C14" s="2" t="n">
         <v>1537</v>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -948,7 +948,7 @@
       <c r="C15" s="2" t="n">
         <v>298.32</v>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -979,7 +979,7 @@
       <c r="C16" s="2" t="n">
         <v>31.88</v>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1010,7 +1010,7 @@
       <c r="C17" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1041,7 +1041,7 @@
       <c r="C18" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1072,7 +1072,7 @@
       <c r="C19" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1103,7 +1103,7 @@
       <c r="C20" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1134,7 +1134,7 @@
       <c r="C21" s="2" t="n">
         <v>878</v>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>נמצא חלקי (פוליסה)</t>
         </is>
@@ -1169,7 +1169,7 @@
       <c r="C22" s="2" t="n">
         <v>2179.25</v>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>נמצא חלקי (פוליסה)</t>
         </is>
@@ -1204,7 +1204,7 @@
       <c r="C23" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>נמצא חלקי (בעמלות לבדוק)</t>
         </is>
@@ -1239,7 +1239,7 @@
       <c r="C24" s="2" t="n">
         <v>8322</v>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1306,7 +1306,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>חשבונית מס קבלה על העברה של 3,983 ₪ מ-15/07 (4,142 ₪ מ-13/10 כבר סגורה בחשבונית 3084)</t>
+          <t>אין. 3,983 ₪ סגורה בקבלה 3067 (פער 2 ₪ מוסבר) ו-4,142 ₪ בקבלה 3084</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mika 3,983 matched to receipt 3085
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vhYGPaAM74nnJetAhxgmr
</commit_message>
<xml_diff>
--- a/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
+++ b/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
@@ -589,22 +589,22 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>נמצא (חשבונית הועלתה לשיחה, פער של 2 ₪)</t>
+          <t>נמצא (חשבונית הועלתה לשיחה)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>חשבונית מס קבלה 3067 מ-17/06/26: 3,981 ₪, על חשבון עסקה 7057 (שירותי משרד מאי). בבנק רשומים 3,983 ₪, כלומר פער של 2 ₪. לפי ההנחיה, זו החשבונית המתאימה והפער הוא טעות. בקבלה עצמה רשום תשלום בהעברה ב-17/06 ולא ב-15/07.</t>
+          <t>חשבונית מס קבלה 3085 מ-14/10/26: 3,983 ₪ (3,375.40 + מע"מ 18%, 607.57 + עיגול 0.03). על חשבון עסקה 7062 (שירותי משרד יוני), ושולמה בהעברה בנקאית ב-15/07/2026. הסכום והתאריך תואמים להעברה. הקבלה 3067 (3,981 ₪, 17/06) היא על חודש מאי ואינה קשורה להעברה הזו.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>קובץ: InvoiceReceipt_3067.pdf</t>
+          <t>קובץ: InvoiceReceipt_3085_source.pdf</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>לא ידוע. 3067 הופיעה בדרייב ב-21/06, ולא נבדק אם נשלחה</t>
+          <t>לא (הופקה ב-14/10, אחרי המשלוח האחרון ב-07/09)</t>
         </is>
       </c>
     </row>
@@ -1306,7 +1306,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>אין. 3,983 ₪ סגורה בקבלה 3067 (פער 2 ₪ מוסבר) ו-4,142 ₪ בקבלה 3084</t>
+          <t>אין. 3,983 ₪ סגורה בקבלה 3085 ו-4,142 ₪ בקבלה 3084</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hatacot rows: findings from emails and Drive
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vhYGPaAM74nnJetAhxgmr
</commit_message>
<xml_diff>
--- a/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
+++ b/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
@@ -50,12 +50,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -659,18 +659,22 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>לא נמצא</t>
+          <t>נמצא חלקי (לבדוק)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>אין בתיבה מסמך על 385 ₪. נמצאו רק: חשבונית 650922 (05/08), קבלות 241875 (05/08) ו-242606 (27/08), וחשבונית 655014 (06/10). לא ניתן לקרוא את תוכן ה-PDF מהמייל, ולכן אי אפשר לשלול שאחת הקבלות היא על 385 ₪.</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr"/>
+          <t>ב-21/06 חן וקנין (גבייה) כתבה: חשבונית 648740 היא על 296 ₪ וההעברה היא 385 ₪, ושאלה אם להשאיר את ההפרש כיתרת זכות. מרגלית אישרה. ב-24/06 נשלחו חשבונית 648740 (296 ₪, הופקה 24/06) וקבלות 240616 ו-240617. סכומי שתי הקבלות לא נקראו (נשלחו כקובץ מצורף במייל). לכן לא אומת איזו קבלה מתאימה לכל אחת משתי ההעברות של 385 ₪. בתגובה כתבה 'הועבר להנה"ש לסגירה'.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>שרשור 21/06: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1867699052471016506 | קבלה 240616: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1868865804863124827 | קבלה 240617: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1868865821241131774 | חשבונית 648740: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1868865831089476373</t>
+        </is>
+      </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>הקבלות 241875, 242606 וחשבונית 650922 נשלחו (07/09/26)</t>
+          <t>לא ידוע. הקבלות והחשבונית הונפקו ב-24/06, ולא נבדק אם נכללו במשלוחי מאי-יוני (14/07)</t>
         </is>
       </c>
     </row>
@@ -682,23 +686,27 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>15/07/26</t>
+          <t>24/06/26</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>375</v>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>לא נמצא</t>
+        <v>296</v>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>נמצא (חשבונית בדרייב)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>אין מסמך על 375 ₪. ראו הערה בשורה הקודמת.</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr"/>
+          <t>חשבונית מס 648740 מ-24/06/26: 296 ₪ כולל מע"מ (250.85 + 45.15). שולמה, לפי חן וקנין, מההעברה של 385 ₪ מ-17/06. נשאר 89 ₪ יתרת זכות. לכן אין תשלום של 296 ₪ בבנק.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>קובץ בדרייב: 648740.pdf. מייל: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1868865831089476373</t>
+        </is>
+      </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
           <t>לא ידוע</t>
@@ -708,65 +716,65 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>קבוצת העתקות (בירור)</t>
+          <t>קבוצת העתקות</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>12/10/26</t>
+          <t>15/07/26</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>296</v>
+        <v>375</v>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>נמצא קשור (לבדוק)</t>
+          <t>נמצא</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>קבלה 244052 התקבלה ב-14/10/26 מ-account3@hatacot.com, כנראה על תשלום 296 ₪ (הסכום לא אומת, צריך לפתוח את ה-PDF). בנוסף, ב-13/10 קבוצת העתקות כתבה שחשבונית 655014 כבר שולמה (קבלה 243829 מ-06/10) והורתה להשאיר את ה-453 ₪ כיתרת זכות. לכן 453 ₪ הם כנראה תשלום עודף שנשאר בזכות ולא תשלום כפול שצריך להחזיר.</t>
+          <t>קבלה 241875 מ-05/08/26: 375 ₪, העברה בנקאית ב-15/07/26, על חשבונית מס 650922 (375 ₪ כולל מע"מ). קבלה 242606 מ-27/08/26 (חנן פישר) היא על 375 ₪ נוספים, העברה מ-06/08/26, עם הערה שהחשבונית כבר שולמה בקבלה 241875. כלומר ייתכן תשלום כפול של 375 ₪ על חשבונית 650922, וכדאי לבקש מקבוצת העתקות יתרת זכות או החזר.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>קבלה 244052: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1879008335247248271 | שרשור 655014: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1878914172447810884</t>
+          <t>קבלה 241875: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1872671606267840776 | חשבונית 650922: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1872671638307010028 | קבלה 242606: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1874673028150340570</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>לא (אחרי 07/09/26)</t>
+          <t>כן. 650922, 241875 ו-242606 נשלחו בחלקים 1-5 (07/09/26)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>גלקסי דיגיטל / מגיק</t>
+          <t>קבוצת העתקות (בירור)</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>13/10/26</t>
+          <t>12/10/26</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>608</v>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>נמצא (סביר, הסכום לא אומת)</t>
+        <v>296</v>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>נמצא חלקי (לבדוק)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>חשבונית מס קבלה דיגיטלית 4-152694 לחודש 10.2026, התקבלה ב-18/10/26 מ-galexiris@gmail.com. נשלחה בעקבות בקשת הקבלה מ-13/10 (חשבון 2-230993). הסכום בתוך ה-PDF לא נקרא.</t>
+          <t>10/09: 453 ₪ נסגרה בקבלה 243829 (06/10/26, העברה מ-10/09, חשבונית 655014). ב-13/10 מרגלית שלחה אישור על העברה של 453 ₪ נוספים ב-12/10 (אסמכתא 825, לחשבונית 655014 ששולמה כבר). חן וקנין כתבה ב-13/10 ש-655014 כבר שולמה ושלהשאיר את הסכום ביתרת זכות. ב-14/10 נשלחה קבלה 244052, והסכום שלה לא נקרא. בטבלת הבנק רשום 296 ₪ ולא 453 ₪, כלומר יש פער בין אישור ההעברה לסכום בבנק. כדאי לבדוק בבנק מה הסכום האמיתי של ההעברה מ-12/10, ולוודא שהקבלה 244052 תואמת לו.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>קבלה: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1879375782021146883 | בקשה: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1878913627659785233</t>
+          <t>הודעת הגבייה: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1878914172447810884 | קבלה 244052: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1879008335247248271 | קבלה 243829: קובץ בדרייב 243829.pdf</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -778,66 +786,70 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>דה קרינה אינטרנט</t>
+          <t>גלקסי דיגיטל / מגיק</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>29/03/26</t>
+          <t>13/10/26</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>350</v>
+        <v>608</v>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>נמצא (בתיבה)</t>
+          <t>נמצא (סביר, הסכום לא אומת)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>חשבונית מס קבלה מ-דה קרינה תעשיות מזון, 29/03/26, דרך PayPlus (הזמנה 7689, מארז שוקולד 350 ₪).</t>
+          <t>חשבונית מס קבלה דיגיטלית 4-152694 לחודש 10.2026, התקבלה ב-18/10/26 מ-galexiris@gmail.com. נשלחה בעקבות בקשת הקבלה מ-13/10 (חשבון 2-230993). הסכום בתוך ה-PDF לא נקרא.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>מייל PayPlus: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1860997030646850739 | אישור הזמנה: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1860996996412043646</t>
+          <t>קבלה: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1879375782021146883 | בקשה: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1878913627659785233</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>לא ידוע. החלקים של מרץ-אפריל נשלחו ב-11/05/26, ללא בדיקה של תוכן הקבצים</t>
+          <t>לא (אחרי 07/09/26)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>טורבו קלין</t>
+          <t>דה קרינה אינטרנט</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>27/07/26</t>
+          <t>29/03/26</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>150</v>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>לא נמצא</t>
+        <v>350</v>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>נמצא (בתיבה)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>אין חשבונית. בדרייב קבלות טורבו של 02/07 (140), 19/04 (145) ו-26/03 (260) בלבד.</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr"/>
+          <t>חשבונית מס קבלה מ-דה קרינה תעשיות מזון, 29/03/26, דרך PayPlus (הזמנה 7689, מארז שוקולד 350 ₪).</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>מייל PayPlus: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1860997030646850739 | אישור הזמנה: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1860996996412043646</t>
+        </is>
+      </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>קבלת 02/07 נשלחה, אבל היא לא על 150 ₪</t>
+          <t>לא ידוע. החלקים של מרץ-אפריל נשלחו ב-11/05/26, ללא בדיקה של תוכן הקבצים</t>
         </is>
       </c>
     </row>
@@ -849,51 +861,51 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>30/08/26</t>
+          <t>27/07/26</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>130</v>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
+        <v>150</v>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>אין חשבונית.</t>
+          <t>אין חשבונית. בדרייב קבלות טורבו של 02/07 (140), 19/04 (145) ו-26/03 (260) בלבד.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr"/>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>קבלת 02/07 נשלחה, אבל היא לא על 150 ₪</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>שליחויות NOW</t>
+          <t>טורבו קלין</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>13/10/26</t>
+          <t>30/08/26</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
         <v>130</v>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>אין מסמך. הקודמת בתיבה: 103871 (31/07/26, 236 ₪), נשלחה. חיפוש המספרים 103834 ו-103854 לא החזיר תוצאות במייל.</t>
+          <t>אין חשבונית.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr"/>
@@ -906,25 +918,25 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>rentalcars</t>
+          <t>שליחויות NOW</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>05/10/26</t>
+          <t>13/10/26</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>1537</v>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
+        <v>130</v>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>חיפוש 'rentalcars' ו-733336639 לא החזיר שום מייל בתיבת המשרד (גם לא אישור הזמנה). אישור ההזמנה ככל הנראה בתיבה של נועם.</t>
+          <t>אין מסמך. הקודמת בתיבה: 103871 (31/07/26, 236 ₪), נשלחה. חיפוש המספרים 103834 ו-103854 לא החזיר תוצאות במייל.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr"/>
@@ -937,25 +949,25 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>notion</t>
+          <t>rentalcars</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>22/09/26</t>
+          <t>05/10/26</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>298.32</v>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
+        <v>1537</v>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>אין מייל מ-Notion בתיבה.</t>
+          <t>חיפוש 'rentalcars' ו-733336639 לא החזיר שום מייל בתיבת המשרד (גם לא אישור הזמנה). אישור ההזמנה ככל הנראה בתיבה של נועם.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr"/>
@@ -968,25 +980,25 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>הוט מובייל</t>
+          <t>notion</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>21/09/26</t>
+          <t>22/09/26</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>31.88</v>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
+        <v>298.32</v>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>אין מייל חשבונית מהוט מובייל. נמצאה רק הצעת מחיר מ-27/07/25.</t>
+          <t>אין מייל מ-Notion בתיבה.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr"/>
@@ -999,25 +1011,25 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>שטיפת האחים</t>
+          <t>הוט מובייל</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>05/10/26</t>
+          <t>21/09/26</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>80</v>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
+        <v>31.88</v>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>אין מסמך.</t>
+          <t>אין מייל חשבונית מהוט מובייל. נמצאה רק הצעת מחיר מ-27/07/25.</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr"/>
@@ -1030,18 +1042,18 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>חניון הרצליה</t>
+          <t>שטיפת האחים</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>18/09/26</t>
+          <t>05/10/26</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
+        <v>80</v>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1061,18 +1073,18 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>חניון בקר</t>
+          <t>חניון הרצליה</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>04/10/26</t>
+          <t>18/09/26</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
+        <v>24</v>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1092,25 +1104,25 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>סנטרל פארק</t>
+          <t>חניון בקר</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>06/10/26</t>
+          <t>04/10/26</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
+        <v>45</v>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>אין מסמך. קבלה קודמת של סנטרל פארק (22/07, 27.14 ₪) נשלחה ביולי-אוגוסט.</t>
+          <t>אין מסמך.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr"/>
@@ -1123,35 +1135,31 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>כלל ביטוח</t>
+          <t>סנטרל פארק</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>28/06/26</t>
+          <t>06/10/26</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>878</v>
+        <v>24</v>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>נמצא חלקי (פוליסה)</t>
+          <t>לא נמצא</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>ב-11/06/26 אודיה גדסי (eshkol4u, ביטוח עסקים) שלחה העתקי פוליסות מחודשות: ביטוח משרד, תכולה, צד ג' ועוד. בדרייב: 'אודיה גדסי - פוליסה 54057121100.pdf'. לא ברור איזו פוליסה מתאימה ל-878 ₪ ולחיובים של 2,179.25 ₪, כי סכומי הפוליסות לא נקראו.</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>שרשור פוליסות: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1866705501130367275</t>
-        </is>
-      </c>
+          <t>אין מסמך. קבלה קודמת של סנטרל פארק (22/07, 27.14 ₪) נשלחה ביולי-אוגוסט.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr"/>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>לא ידוע</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
@@ -1163,20 +1171,20 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>28/6, 27/7, 26/8, 27/9</t>
+          <t>28/06/26</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>2179.25</v>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
+        <v>878</v>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>נמצא חלקי (פוליסה)</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>אותו שרשור פוליסות. 4 חיובים בסכום זהה, כנראה תשלומים על פוליסה מחודשת (חידוש ב-06/2026 בכמה תשלומים).</t>
+          <t>ב-11/06/26 אודיה גדסי (eshkol4u, ביטוח עסקים) שלחה העתקי פוליסות מחודשות: ביטוח משרד, תכולה, צד ג' ועוד. בדרייב: 'אודיה גדסי - פוליסה 54057121100.pdf'. לא ברור איזו פוליסה מתאימה ל-878 ₪ ולחיובים של 2,179.25 ₪, כי סכומי הפוליסות לא נקראו.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1193,64 +1201,99 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>רב חסד</t>
+          <t>כלל ביטוח</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>1-9/2026, חודשי</t>
+          <t>28/6, 27/7, 26/8, 27/9</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>120</v>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>נמצא חלקי (בעמלות לבדוק)</t>
+        <v>2179.25</v>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>נמצא חלקי (פוליסה)</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>קבלות על תרומות מגיעות לתיבה כהעברות מנועם ממוסדות 'משכן מנחם חב"ד' (30004153, 30004658, 30005166), ו'ישמח ישראל' (213920, 213958, 770804). לא נמצא מוסד בשם 'רב חסד'. ב-07/09/26 נשלחו לפנינה 26 קבלות תרומה (סעיף 46). פנינה ענתה שאפשר גם דרך ביזיבוקס.</t>
+          <t>אותו שרשור פוליסות. 4 חיובים בסכום זהה, כנראה תשלומים על פוליסה מחודשת (חידוש ב-06/2026 בכמה תשלומים).</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>שליחה לפנינה: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1875675882405265785</t>
+          <t>שרשור פוליסות: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1866705501130367275</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>26 קבלות נשלחו לפנינה (לא לביזיבוקס). הקבלות הספציפיות על 120 ₪ לא אומתו</t>
+          <t>לא ידוע</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
+          <t>רב חסד</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>1-9/2026, חודשי</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>נמצא חלקי (בעמלות לבדוק)</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>קבלות על תרומות מגיעות לתיבה כהעברות מנועם ממוסדות 'משכן מנחם חב"ד' (30004153, 30004658, 30005166), ו'ישמח ישראל' (213920, 213958, 770804). לא נמצא מוסד בשם 'רב חסד'. ב-07/09/26 נשלחו לפנינה 26 קבלות תרומה (סעיף 46). פנינה ענתה שאפשר גם דרך ביזיבוקס.</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>שליחה לפנינה: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1875675882405265785</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>26 קבלות נשלחו לפנינה (לא לביזיבוקס). הקבלות הספציפיות על 120 ₪ לא אומתו</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
           <t>אוראגן תירוש (לבדוק)</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>20/03/26</t>
         </is>
       </c>
-      <c r="C24" s="2" t="n">
+      <c r="C25" s="2" t="n">
         <v>8322</v>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>חיפוש 'תירוש' / 'tiroche' לא החזיר מייל בתיבת המשרד. החשבונית המתוקנת מ-keren.m@tiroche.co.il לא נמצאת כאן, ולכן אי אפשר לאמת אם היא סופית או טיוטה.</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr"/>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr"/>
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>לא ידוע</t>
         </is>
@@ -1318,7 +1361,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>קבלות/חשבוניות על 385 ₪ x2 (17/06), 375 ₪ (15/07), ואישור שקבלה 244052 היא על 296 ₪</t>
+          <t>אימות סכומי הקבלות 240616 ו-240617 (ההעברות של 385 ₪), סכום קבלה 244052, ויתרות הזכות: 89 ₪ מיוני, 453 ₪ מ-12/10 ו-375 ₪ מ-06/08 (כפול על חשבונית 650922). האם לקזז מחשבוניות עתידיות או להחזיר</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hatacot receipt 244052 (453, duplicate, credit balance)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vhYGPaAM74nnJetAhxgmr
</commit_message>
<xml_diff>
--- a/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
+++ b/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
@@ -762,19 +762,19 @@
       <c r="C9" s="2" t="n">
         <v>296</v>
       </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>נמצא חלקי (לבדוק)</t>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>נמצא (קבלה הועלתה לשיחה, סכום שונה)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>10/09: 453 ₪ נסגרה בקבלה 243829 (06/10/26, העברה מ-10/09, חשבונית 655014). ב-13/10 מרגלית שלחה אישור על העברה של 453 ₪ נוספים ב-12/10 (אסמכתא 825, לחשבונית 655014 ששולמה כבר). חן וקנין כתבה ב-13/10 ש-655014 כבר שולמה ושלהשאיר את הסכום ביתרת זכות. ב-14/10 נשלחה קבלה 244052, והסכום שלה לא נקרא. בטבלת הבנק רשום 296 ₪ ולא 453 ₪, כלומר יש פער בין אישור ההעברה לסכום בבנק. כדאי לבדוק בבנק מה הסכום האמיתי של ההעברה מ-12/10, ולוודא שהקבלה 244052 תואמת לו.</t>
+          <t>קבלה 244052 מ-14/10/26: 453 ₪, העברה בנקאית מ-12/10/26. בקבלה כתוב 'כפילות, ביתרת זכות-לקוח/חן', כלומר זה תשלום כפול על חשבונית 655014 (שכבר שולמה ב-10/09 בקבלה 243829), והסכום נשאר אצלם כיתרת זכות. הסכום בקבלה (453 ₪) שונה מהסכום בטבלת הבנק (296 ₪), כך שצריך לבדוק בבנק מה נגבה בפועל ב-12/10.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>הודעת הגבייה: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1878914172447810884 | קבלה 244052: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1879008335247248271 | קבלה 243829: קובץ בדרייב 243829.pdf</t>
+          <t>קובץ: 244052.pdf | הודעת הגבייה: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1878914172447810884</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -1361,7 +1361,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>אימות סכומי הקבלות 240616 ו-240617 (ההעברות של 385 ₪), סכום קבלה 244052, ויתרות הזכות: 89 ₪ מיוני, 453 ₪ מ-12/10 ו-375 ₪ מ-06/08 (כפול על חשבונית 650922). האם לקזז מחשבוניות עתידיות או להחזיר</t>
+          <t>אימות סכומי הקבלות 240616 ו-240617 (ההעברות של 385 ₪), ויתרות הזכות: 89 ₪ מיוני, 453 ₪ מ-12/10 ו-375 ₪ מ-06/08 (כפול על חשבונית 650922). האם לקזז מחשבוניות עתידיות או להחזיר</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hatacot receipt 240617 (385 on 17/06)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vhYGPaAM74nnJetAhxgmr
</commit_message>
<xml_diff>
--- a/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
+++ b/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
@@ -50,12 +50,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -657,14 +657,14 @@
       <c r="C6" s="2" t="n">
         <v>385</v>
       </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>נמצא חלקי (לבדוק)</t>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>נמצא (העברה אחת מאומתת, השנייה כנראה)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>ב-21/06 חן וקנין (גבייה) כתבה: חשבונית 648740 היא על 296 ₪ וההעברה היא 385 ₪, ושאלה אם להשאיר את ההפרש כיתרת זכות. מרגלית אישרה. ב-24/06 נשלחו חשבונית 648740 (296 ₪, הופקה 24/06) וקבלות 240616 ו-240617. סכומי שתי הקבלות לא נקראו (נשלחו כקובץ מצורף במייל). לכן לא אומת איזו קבלה מתאימה לכל אחת משתי ההעברות של 385 ₪. בתגובה כתבה 'הועבר להנה"ש לסגירה'.</t>
+          <t>קבלה 240617 מ-24/06/26: 385 ₪, העברה בנקאית מ-17/06/26 (הועלתה לשיחה וקראתי אותה). קבלה 240616 נשלחה באותו יום ובאותו מייל, וכנראה מכסה את ההעברה השנייה של 385 ₪ מ-17/06, אבל הסכום שלה לא נקרא. ב-21/06 חן וקנין כתבה שחשבונית 648740 היא על 296 ₪ ושההעברה (385 ₪) עודפת, והשאירה את ההפרש (89 ₪) כיתרת זכות. אם שתי ההעברות הן של 385 ₪, יש אצלם בנוסף 385 ₪ בזכות, והשאלה אם זה כך נשארת פתוחה.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -727,7 +727,7 @@
       <c r="C8" s="2" t="n">
         <v>375</v>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>נמצא</t>
         </is>
@@ -867,7 +867,7 @@
       <c r="C12" s="2" t="n">
         <v>150</v>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -898,7 +898,7 @@
       <c r="C13" s="2" t="n">
         <v>130</v>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -929,7 +929,7 @@
       <c r="C14" s="2" t="n">
         <v>130</v>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -960,7 +960,7 @@
       <c r="C15" s="2" t="n">
         <v>1537</v>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -991,7 +991,7 @@
       <c r="C16" s="2" t="n">
         <v>298.32</v>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1022,7 +1022,7 @@
       <c r="C17" s="2" t="n">
         <v>31.88</v>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1053,7 +1053,7 @@
       <c r="C18" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1084,7 +1084,7 @@
       <c r="C19" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1115,7 +1115,7 @@
       <c r="C20" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1146,7 +1146,7 @@
       <c r="C21" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1177,7 +1177,7 @@
       <c r="C22" s="2" t="n">
         <v>878</v>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>נמצא חלקי (פוליסה)</t>
         </is>
@@ -1212,7 +1212,7 @@
       <c r="C23" s="2" t="n">
         <v>2179.25</v>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>נמצא חלקי (פוליסה)</t>
         </is>
@@ -1247,7 +1247,7 @@
       <c r="C24" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>נמצא חלקי (בעמלות לבדוק)</t>
         </is>
@@ -1282,7 +1282,7 @@
       <c r="C25" s="2" t="n">
         <v>8322</v>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1361,7 +1361,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>אימות סכומי הקבלות 240616 ו-240617 (ההעברות של 385 ₪), ויתרות הזכות: 89 ₪ מיוני, 453 ₪ מ-12/10 ו-375 ₪ מ-06/08 (כפול על חשבונית 650922). האם לקזז מחשבוניות עתידיות או להחזיר</t>
+          <t>אימות סכום קבלה 240616 (ההעברה השנייה של 385 ₪), ויתרות הזכות: 89 ₪ מיוני, 453 ₪ מ-12/10 ו-375 ₪ מ-06/08 (כפול על חשבונית 650922). האם לקזז מחשבוניות עתידיות או להחזיר</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hatacot receipt 240616: both 385 transfers covered
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vhYGPaAM74nnJetAhxgmr
</commit_message>
<xml_diff>
--- a/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
+++ b/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
@@ -659,12 +659,12 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>נמצא (העברה אחת מאומתת, השנייה כנראה)</t>
+          <t>נמצא (שתי ההעברות, הקבלות הועלו לשיחה)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>קבלה 240617 מ-24/06/26: 385 ₪, העברה בנקאית מ-17/06/26 (הועלתה לשיחה וקראתי אותה). קבלה 240616 נשלחה באותו יום ובאותו מייל, וכנראה מכסה את ההעברה השנייה של 385 ₪ מ-17/06, אבל הסכום שלה לא נקרא. ב-21/06 חן וקנין כתבה שחשבונית 648740 היא על 296 ₪ ושההעברה (385 ₪) עודפת, והשאירה את ההפרש (89 ₪) כיתרת זכות. אם שתי ההעברות הן של 385 ₪, יש אצלם בנוסף 385 ₪ בזכות, והשאלה אם זה כך נשארת פתוחה.</t>
+          <t>קבלות 240616 ו-240617, שתיהן מ-24/06/26: כל אחת 385 ₪, העברה בנקאית מ-17/06/26. בכך שתי ההעברות מכוסות. ב-21/06 חן וקנין כתבה שחשבונית 648740 היא על 296 ₪ ושההעברה (385 ₪) עודפת, והשאירה כיתרת זכות. כיוון ששולמו 770 ₪ על חשבונית של 296 ₪, נשארה אצלם יתרת זכות של כ-474 ₪. לא ברור אם היא משקפת תשלום כפול או תשלום מראש, וכדאי לאמת מולם.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -1361,7 +1361,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>אימות סכום קבלה 240616 (ההעברה השנייה של 385 ₪), ויתרות הזכות: 89 ₪ מיוני, 453 ₪ מ-12/10 ו-375 ₪ מ-06/08 (כפול על חשבונית 650922). האם לקזז מחשבוניות עתידיות או להחזיר</t>
+          <t>אישור יתרות הזכות: 474 ₪ מיוני (770 ₪ שולמו על חשבונית של 296 ₪), 453 ₪ מ-12/10 ו-375 ₪ מ-06/08 (כפול על חשבונית 650922). האם לקזז מחשבוניות עתידיות או להחזיר</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hatacot 12/10: bank shows 453, matches receipt 244052
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vhYGPaAM74nnJetAhxgmr
</commit_message>
<xml_diff>
--- a/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
+++ b/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
@@ -760,21 +760,21 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>296</v>
+        <v>453</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>נמצא (קבלה הועלתה לשיחה, סכום שונה)</t>
+          <t>נמצא (נסגר, תיקון סכום)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>קבלה 244052 מ-14/10/26: 453 ₪, העברה בנקאית מ-12/10/26. בקבלה כתוב 'כפילות, ביתרת זכות-לקוח/חן', כלומר זה תשלום כפול על חשבונית 655014 (שכבר שולמה ב-10/09 בקבלה 243829), והסכום נשאר אצלם כיתרת זכות. הסכום בקבלה (453 ₪) שונה מהסכום בטבלת הבנק (296 ₪), כך שצריך לבדוק בבנק מה נגבה בפועל ב-12/10.</t>
+          <t>בבנק מרכנתיל דיסקונט נרשמה ב-12/10/26 העברה באינטרנט של 453 ₪ לקבוצת העתקות, בהערה 'חן 655014' (צילום מסך מהבנק). זה תואם לקבלה 244052 (453 ₪, 14/10/26) ולאישור ההעברה שנשלח ב-13/10. כלומר הסכום בטבלת התנועות הפתוחות (296 ₪) היה שגוי, והסכום הנכון הוא 453 ₪. זה תשלום כפול על חשבונית 655014, ששולמה ב-10/09 (קבלה 243829). הסכום נשאר אצל קבוצת העתקות כיתרת זכות.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>קובץ: 244052.pdf | הודעת הגבייה: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1878914172447810884</t>
+          <t>קבלה: קובץ 244052.pdf | הודעת הגבייה: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1878914172447810884</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Galaxy invoice 4-152694 verified: 608
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vhYGPaAM74nnJetAhxgmr
</commit_message>
<xml_diff>
--- a/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
+++ b/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
@@ -799,12 +799,12 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>נמצא (סביר, הסכום לא אומת)</t>
+          <t>נמצא (חשבונית הועלתה לשיחה)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>חשבונית מס קבלה דיגיטלית 4-152694 לחודש 10.2026, התקבלה ב-18/10/26 מ-galexiris@gmail.com. נשלחה בעקבות בקשת הקבלה מ-13/10 (חשבון 2-230993). הסכום בתוך ה-PDF לא נקרא.</t>
+          <t>חשבונית מס/קבלה 4-152694 מ-18/10/26 (galexiris@gmail.com): 608 ₪ (515.25 + מע"מ 18%, 92.75), תשלום בהעברה מ-13/10/26, עבור חשבון 2-230993 מ-30/09/26. הסכום והתאריך תואמים להעברה.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1310,7 +1310,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -1425,18 +1425,6 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>גלקסי דיגיטל</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>אימות שחשבונית 4-152694 היא על 608 ₪</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Clal rows: professional liability policy matches 4x2179.25
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vhYGPaAM74nnJetAhxgmr
</commit_message>
<xml_diff>
--- a/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
+++ b/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
@@ -1179,17 +1179,17 @@
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>נמצא חלקי (פוליסה)</t>
+          <t>נמצא חלקי (פוליסה לא נקראה)</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>ב-11/06/26 אודיה גדסי (eshkol4u, ביטוח עסקים) שלחה העתקי פוליסות מחודשות: ביטוח משרד, תכולה, צד ג' ועוד. בדרייב: 'אודיה גדסי - פוליסה 54057121100.pdf'. לא ברור איזו פוליסה מתאימה ל-878 ₪ ולחיובים של 2,179.25 ₪, כי סכומי הפוליסות לא נקראו.</t>
+          <t>ב-11/06/26 אודיה גדסי שלחה שתי פוליסות מחודשות: 64057121100 (אחריות מקצועית) ו-64069979800 (ביטוח משרד: תכולה, צד ג', חבות מעבידים). החיוב של 878 ₪ כנראה שייך לפוליסת המשרד 64069979800, אבל הפוליסה הזו לא נמצאת בדרייב ולא נקראה, ולכן הסכום לא אומת.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>שרשור פוליסות: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1866705501130367275</t>
+          <t>שרשור הפוליסות: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1866705501130367275</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -1212,19 +1212,19 @@
       <c r="C23" s="2" t="n">
         <v>2179.25</v>
       </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>נמצא חלקי (פוליסה)</t>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>נמצא (פוליסה בדרייב)</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>אותו שרשור פוליסות. 4 חיובים בסכום זהה, כנראה תשלומים על פוליסה מחודשת (חידוש ב-06/2026 בכמה תשלומים).</t>
+          <t>פוליסה 64057121100 (אחריות מקצועית, כלל ביטוח דרך אשכול 4U): תקופה 01/06/2026-31/05/2027, פרמיה נטו 7,580 ₪, סה"כ 8,717 ₪ כולל תוספת. 4 x 2,179.25 = 8,717 ₪, לכן ארבעת החיובים הם תשלומי הפוליסה בארבעה תשלומים. הפוליסה נמצאת בדרייב.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>שרשור פוליסות: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1866705501130367275</t>
+          <t>פוליסה בדרייב: אודיה גדסי - פוליסה 64057121100.pdf | שרשור: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1866705501130367275</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -1421,7 +1421,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>פירוט איזו פוליסה מתאימה ל-878 ₪ (28/06) ול-2,179.25 ₪ x4</t>
+          <t>אישור שהחיוב של 878 ₪ (28/06) הוא תשלום על פוליסת המשרד 64069979800, וכמה תשלומים נוספים צפויים</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Clal 878 matched to office policy 64069979800
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vhYGPaAM74nnJetAhxgmr
</commit_message>
<xml_diff>
--- a/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
+++ b/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
@@ -1177,19 +1177,19 @@
       <c r="C22" s="2" t="n">
         <v>878</v>
       </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>נמצא חלקי (פוליסה לא נקראה)</t>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>נמצא (פוליסה הועלתה לשיחה)</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>ב-11/06/26 אודיה גדסי שלחה שתי פוליסות מחודשות: 64057121100 (אחריות מקצועית) ו-64069979800 (ביטוח משרד: תכולה, צד ג', חבות מעבידים). החיוב של 878 ₪ כנראה שייך לפוליסת המשרד 64069979800, אבל הפוליסה הזו לא נמצאת בדרייב ולא נקראה, ולכן הסכום לא אומת.</t>
+          <t>פוליסה 64069979800 (ביטוח משרד, כלל ביטוח דרך אשכול 4U): תקופה 01/06/2026-31/05/2027, פרמיה שנתית 878 ₪ בתשלום אחד, בכרטיס אשראי בהוראת קבע. זהה לחיוב מ-28/06 ולכן הוא התשלום השנתי על הפוליסה. הפוליסה נשלחה במייל מ-11/06/26.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>שרשור הפוליסות: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1866705501130367275</t>
+          <t>שרשור הפוליסות: https://mail.google.com/mail/?authuser=office.noamsander@gmail.com#all/thread-f:1866705501130367275 | קובץ: פוליסה 64069979800.pdf</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -1421,7 +1421,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>אישור שהחיוב של 878 ₪ (28/06) הוא תשלום על פוליסת המשרד 64069979800, וכמה תשלומים נוספים צפויים</t>
+          <t>אין. שני החיובים של כלל סגורים בפוליסות (878 ₪ בפוליסה 64069979800 ו-8,717 ₪ בפוליסה 64057121100)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
NOW invoice 103910 matches 130 on 13/10
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vhYGPaAM74nnJetAhxgmr
</commit_message>
<xml_diff>
--- a/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
+++ b/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
@@ -929,20 +929,24 @@
       <c r="C14" s="2" t="n">
         <v>130</v>
       </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>לא נמצא</t>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>נמצא (חשבונית הועלתה לשיחה)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>אין מסמך. הקודמת בתיבה: 103871 (31/07/26, 236 ₪), נשלחה. חיפוש המספרים 103834 ו-103854 לא החזיר תוצאות במייל.</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr"/>
+          <t>חשבונית מס 103910 מ-30/09/2026: 130 ₪ (110.17 + מע"מ 18%, 19.83). משלוח אחד, מגיזה ברזל 4 רמת החייל אל מרגלית בפתח תקווה. הסכום תואם לחיוב מ-13/10. בנוסף הועלתה חשבונית 103835 מ-31/05/2026 על 260 ₪ (שני משלוחים), שאינה קשורה לחיוב הזה.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>קבצים: doc_31597115_51545_inv103910.pdf, doc_31597115_50993_inv103835.pdf</t>
+        </is>
+      </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>לא (אחרי 07/09/26)</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1314,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -1380,46 +1384,34 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>שליחויות NOW</t>
+          <t>חניון הרצליה, חניון בקר, שטיפת האחים</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>חשבונית על 130 ₪ (13/10)</t>
+          <t>קבלות על 24 ₪, 45 ₪, 80 ₪ (או להסיר משיקולי סכום)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>חניון הרצליה, חניון בקר, שטיפת האחים</t>
+          <t>נועם (noamsander@gmail.com)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>קבלות על 24 ₪, 45 ₪, 80 ₪ (או להסיר משיקולי סכום)</t>
+          <t>אישור הזמנה / חשבונית rentalcars 1,537 ₪; חשבונית Notion 298.32 ₪; חשבונית הוט מובייל 31.88 ₪; חשבונית תירוש 8,322 ₪ (מ-keren.m@tiroche.co.il); קבלות 'רב חסד' על 120 ₪ לחודש</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>נועם (noamsander@gmail.com)</t>
+          <t>אודיה גדסי (eshkol4u.co.il)</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>אישור הזמנה / חשבונית rentalcars 1,537 ₪; חשבונית Notion 298.32 ₪; חשבונית הוט מובייל 31.88 ₪; חשבונית תירוש 8,322 ₪ (מ-keren.m@tiroche.co.il); קבלות 'רב חסד' על 120 ₪ לחודש</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>אודיה גדסי (eshkol4u.co.il)</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>אין. שני החיובים של כלל סגורים בפוליסות (878 ₪ בפוליסה 64069979800 ו-8,717 ₪ בפוליסה 64057121100)</t>
         </is>

</xml_diff>

<commit_message>
Add consolidated list of what is still missing
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vhYGPaAM74nnJetAhxgmr
</commit_message>
<xml_diff>
--- a/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
+++ b/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
@@ -7,8 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="תוצאות חיפוש" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מה חסר ממי לבקש" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="רשימת חסרים" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="תוצאות חיפוש" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מה חסר ממי לבקש" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -71,13 +72,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -454,6 +458,896 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>קבוצה</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ספק / לקוח</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>תאריך</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>סכום ₪</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>מה חסר</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>ממי לבקש / מה לעשות</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>א. הוצאות: חשבונית לא נמצאה</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>טורבו קלין</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>27/07/26</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>חשבונית/קבלה על שטיפת רכב</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>טורבו קלין (בטלפון או בוואטסאפ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>א. הוצאות: חשבונית לא נמצאה</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>טורבו קלין</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>30/08/26</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>130</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>חשבונית/קבלה על שטיפת רכב</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>טורבו קלין</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>א. הוצאות: חשבונית לא נמצאה</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>rentalcars</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>05/10/26</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>1537</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>חשבונית/קבלה (נמצא רק אישור הזמנה 733336639, ובמייל המשרד אין אפילו אישור)</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>נועם: חיפוש בתיבה שלו, ואם אין, אתר rentalcars</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>א. הוצאות: חשבונית לא נמצאה</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>notion</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>22/09/26</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>298.32</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>חשבונית</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>נועם / הגדרות החשבון ב-Notion (Billing)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>א. הוצאות: חשבונית לא נמצאה</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>הוט מובייל</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>21/09/26</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>31.88</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>חשבונית</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>נועם / האזור האישי בהוט מובייל</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>א. הוצאות: חשבונית לא נמצאה</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>שטיפת האחים</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>05/10/26</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>קבלה</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>נועם / ספק</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>א. הוצאות: חשבונית לא נמצאה</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>חניון הרצליה</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>18/09/26</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>קבלה</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>נועם / חניון, או להשאיר כהוצאה קטנה ללא קבלה</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>א. הוצאות: חשבונית לא נמצאה</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>חניון בקר</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>04/10/26</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>קבלה</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>נועם / חניון, או להשאיר כהוצאה קטנה ללא קבלה</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>א. הוצאות: חשבונית לא נמצאה</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>סנטרל פארק</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>06/10/26</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>קבלה</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>נועם / חניון, או להשאיר כהוצאה קטנה ללא קבלה</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>א. הוצאות: חשבונית לא נמצאה</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>אוראגן תירוש</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>20/03/26</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>8322</v>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>חשבונית מס סופית (המתוקנת מ-keren.m@tiroche.co.il לא נמצאת בתיבת המשרד, צריך לוודא שאינה טיוטה)</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>נועם / keren.m@tiroche.co.il</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>א. הוצאות: חשבונית לא נמצאה</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>רב חסד (תרומות)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>1-9/2026</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>9 קבלות על תרומה בסעיף 46, 120 ₪ לחודש. לא נמצא מוסד בשם הזה במייל</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>נועם. ייתכן שחלק מהקבלות כבר בתוך 26 הקבלות שנשלחו לפנינה ב-07/09</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>ב. נמצא, ממתין לשליחה לביזיבוקס</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>נחמן כהן</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>15/07, 13/10 x2</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>3540</v>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>חשבוניות 200385, 200389, 200391 (1,180 ₪ כל אחת). לא נשלחו</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>לשלוח לביזיבוקס</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>ב. נמצא, ממתין לשליחה לביזיבוקס</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>מיקה שרותי משרד</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>15/07, 13/10</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>8125</v>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>קבלות 3085 (3,983 ₪) ו-3084 (4,142 ₪)</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>לשלוח לביזיבוקס</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>ב. נמצא, ממתין לשליחה לביזיבוקס</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>קבוצת העתקות</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>17/06 x2, 24/06, 12/10</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>1566</v>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>קבלות 240616 ו-240617 (385 ₪ כל אחת), חשבונית 648740 (296 ₪), קבלה 244052 (453 ₪)</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>לשלוח לביזיבוקס</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>ב. נמצא, ממתין לשליחה לביזיבוקס</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>שליחויות NOW</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>13/10/26</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>130</v>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>חשבונית 103910 מ-30/09/26 (130 ₪). חשבונית 103835 (260 ₪, 31/05/26) לא ידוע אם נשלחה</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>לשלוח לביזיבוקס</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>ב. נמצא, ממתין לשליחה לביזיבוקס</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>גלקסי דיגיטל</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>13/10/26</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>608</v>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>חשבונית מס קבלה 4-152694</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>לשלוח לביזיבוקס</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>ב. נמצא, ממתין לשליחה לביזיבוקס</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>כלל ביטוח</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>28/06 ואילך</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>9595</v>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>פוליסות 64057121100 (8,717 ₪) ו-64069979800 (878 ₪)</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>לשלוח לביזיבוקס</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>ב. נמצא, ממתין לשליחה לביזיבוקס</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>פנגו</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>ספטמבר-אוקטובר</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>פנינה כתבה ב-18/10 שחשבוניות המס של פנגו חסרות. יש כ-18 חיובים של פנגו בכרטיס 1125</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>להוריד חשבונית מרוכזת מהאזור האישי של פנגו ולשלוח לביזיבוקס</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>ג. לבדוק מול הספק</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>קבוצת העתקות</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>12/10, 06/08, 17/06</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>1302</v>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>יתרות זכות: 453 ₪ (תשלום כפול על 655014), 375 ₪ (תשלום כפול על 650922), כ-474 ₪ מיוני. סה"כ כ-1,300 ₪</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>חן וקנין: כרטסת, וקיזוז או החזר (הטיוטה במייל המשרד)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>ג. לבדוק מול הספק</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>אשכול 4U ביטוח</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>30/01, 28/02/26</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>156.91</v>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>חשבוניות 18 (70.91 ₪) ו-182 (86 ₪): לא נמצא חיוב בבנק</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>לבדוק באשראי / לשאול את אשכול 4U איך שולם</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>ג. לבדוק מול הספק</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>גלקסי דיגיטל</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>31/10, 20/11/25</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>חשבונית 723 על 503 ₪ מול העברה של 475 ₪: חסרים 28 ₪</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>לסגור מול גלקסי</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>ד. הכנסות (מהקובץ, לא נחקר בחיפוש)</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>לקוח: לח אחד העם / בן שושן הילה</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>06/07/26</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>10230</v>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>חשבונית הכנסה להעברה</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>להוציא חשבונית הכנסה</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>ד. הכנסות (מהקובץ, לא נחקר בחיפוש)</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>לקוח: מגדלה בע"מ</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>09/10/26 (בקובץ כתוב 1926)</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>15930</v>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>חשבונית הכנסה להעברה</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>להוציא חשבונית הכנסה</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>ד. הכנסות (מהקובץ, לא נחקר בחיפוש)</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>לקוח: מקורון פטיסרי (זיכוי)</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>12/10/26</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>17700</v>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>חשבונית הכנסה להעברה</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>להוציא חשבונית הכנסה</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>ד. הכנסות (מהקובץ, לא נחקר בחיפוש)</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>לקוח: ג'ויה אור</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>23/09/26</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>2950</v>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>חשבונית הכנסה להפקדת שיק (פנינה חזרה על כך ב-18/10)</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>להוציא חשבונית הכנסה</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>ד. הכנסות (מהקובץ, לא נחקר בחיפוש)</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>לקוח: ננוס לאנצ'</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>02/03/26</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="n">
+        <v>7965</v>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>5 חשבוניות מול 4 העברות. שיק 21078 לא הופקד (פנינה, 18/10)</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>לבדוק איזו חשבונית פתוחה, ולהחליט מה לעשות עם השיק</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>ד. הכנסות (מהקובץ, לא נחקר בחיפוש)</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>לקוחות עם יתרה פתוחה</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>שונים</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>מ.ד.ע עזריאלי: חשבונית 20022 (17,700 ₪), שולמו 8,850 ₪ ונשארו 8,850 ₪. ביט.ברידג (קמפינסקי): חשבונית 20044 (11,800 ₪). פיצריה בר דיזנגוף: חשבונית 40150 (9,440 ₪)</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>לברר מול הלקוחות איך ייסגרו היתרות (בהערות בקובץ כתוב 'יודעת')</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>ה. תיקוני רשימה</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>רשימת התנועות הפתוחות</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>12/10/26</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>453</v>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>בקובץ רשום 296 ₪ להעברה מ-12/10 לקבוצת העתקות. בבנק ובקבלה 244052 הסכום הוא 453 ₪</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>לתקן ברשימה לפני שליחה לפנינה</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -467,37 +1361,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>ספק</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>תאריך חיוב</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>סכום ₪</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>נמצא / לא נמצא</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>מה נמצא (תאריך, שולח, נושא)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>קישור למייל</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>נשלח לביזיבוקס?</t>
         </is>
@@ -517,7 +1411,7 @@
       <c r="C2" s="2" t="n">
         <v>1180</v>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>נמצא (כנראה, לפי שתי חשבוניות שהועלו)</t>
         </is>
@@ -552,7 +1446,7 @@
       <c r="C3" s="2" t="n">
         <v>1180</v>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>נמצא (חשבונית הועלתה לשיחה)</t>
         </is>
@@ -587,7 +1481,7 @@
       <c r="C4" s="2" t="n">
         <v>3983</v>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>נמצא (חשבונית הועלתה לשיחה)</t>
         </is>
@@ -622,7 +1516,7 @@
       <c r="C5" s="2" t="n">
         <v>4142</v>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>נמצא (חשבונית הועלתה לשיחה)</t>
         </is>
@@ -657,7 +1551,7 @@
       <c r="C6" s="2" t="n">
         <v>385</v>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>נמצא (שתי ההעברות, הקבלות הועלו לשיחה)</t>
         </is>
@@ -692,7 +1586,7 @@
       <c r="C7" s="2" t="n">
         <v>296</v>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>נמצא (חשבונית בדרייב)</t>
         </is>
@@ -727,7 +1621,7 @@
       <c r="C8" s="2" t="n">
         <v>375</v>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>נמצא</t>
         </is>
@@ -762,7 +1656,7 @@
       <c r="C9" s="2" t="n">
         <v>453</v>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>נמצא (נסגר, תיקון סכום)</t>
         </is>
@@ -797,7 +1691,7 @@
       <c r="C10" s="2" t="n">
         <v>608</v>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>נמצא (חשבונית הועלתה לשיחה)</t>
         </is>
@@ -832,7 +1726,7 @@
       <c r="C11" s="2" t="n">
         <v>350</v>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>נמצא (בתיבה)</t>
         </is>
@@ -867,7 +1761,7 @@
       <c r="C12" s="2" t="n">
         <v>150</v>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -898,7 +1792,7 @@
       <c r="C13" s="2" t="n">
         <v>130</v>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -929,7 +1823,7 @@
       <c r="C14" s="2" t="n">
         <v>130</v>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>נמצא (חשבונית הועלתה לשיחה)</t>
         </is>
@@ -964,7 +1858,7 @@
       <c r="C15" s="2" t="n">
         <v>1537</v>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -995,7 +1889,7 @@
       <c r="C16" s="2" t="n">
         <v>298.32</v>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1026,7 +1920,7 @@
       <c r="C17" s="2" t="n">
         <v>31.88</v>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1057,7 +1951,7 @@
       <c r="C18" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1088,7 +1982,7 @@
       <c r="C19" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1119,7 +2013,7 @@
       <c r="C20" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1150,7 +2044,7 @@
       <c r="C21" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1181,7 +2075,7 @@
       <c r="C22" s="2" t="n">
         <v>878</v>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>נמצא (פוליסה הועלתה לשיחה)</t>
         </is>
@@ -1216,7 +2110,7 @@
       <c r="C23" s="2" t="n">
         <v>2179.25</v>
       </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>נמצא (פוליסה בדרייב)</t>
         </is>
@@ -1251,7 +2145,7 @@
       <c r="C24" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>נמצא חלקי (בעמלות לבדוק)</t>
         </is>
@@ -1286,7 +2180,7 @@
       <c r="C25" s="2" t="n">
         <v>8322</v>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>לא נמצא</t>
         </is>
@@ -1308,7 +2202,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1322,12 +2216,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>ממי לבקש</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>מה לבקש</t>
         </is>

</xml_diff>

<commit_message>
Income section: details from emails
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vhYGPaAM74nnJetAhxgmr
</commit_message>
<xml_diff>
--- a/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
+++ b/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1132,72 +1132,72 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>ד. הכנסות (מהקובץ, לא נחקר בחיפוש)</t>
+          <t>ד. הכנסות</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>לקוח: לח אחד העם / בן שושן הילה</t>
+          <t>מגדלה בע"מ (ח.פ 513781351)</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>06/07/26</t>
+          <t>09/10/26 (בקובץ כתוב 1926)</t>
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>10230</v>
+        <v>15930</v>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>חשבונית הכנסה להעברה</t>
+          <t>חשבון עסקה 1154 נשלח ב-05/10/26: 15,930 ₪ (13,500 + מע"מ), 30% מהעסקה. הלקוח שילם ב-09/10. ב-15/10 מנהלת החשבונות שלהם כתבה שלא התקבלה חשבונית מס, וב-18/10 נשלחה להם חשבונית מס קבלה. נשאר לשלוח את החשבונית לפנינה (דוח הכנסות אוקטובר)</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>להוציא חשבונית הכנסה</t>
+          <t>להעביר לפנינה את חשבונית המס קבלה ששלחת ב-18/10</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>ד. הכנסות (מהקובץ, לא נחקר בחיפוש)</t>
+          <t>ד. הכנסות</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>לקוח: מגדלה בע"מ</t>
+          <t>לח אחד העם / בן שושן הילה</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>09/10/26 (בקובץ כתוב 1926)</t>
+          <t>06/07/26</t>
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>15930</v>
+        <v>10230</v>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>חשבונית הכנסה להעברה</t>
+          <t>לא נמצא במייל מסמך על העברה זו. צריך לברר עבור איזה פרויקט שולם</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>להוציא חשבונית הכנסה</t>
+          <t>לברר מול נעם ולהוציא חשבונית הכנסה</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>ד. הכנסות (מהקובץ, לא נחקר בחיפוש)</t>
+          <t>ד. הכנסות</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>לקוח: מקורון פטיסרי (זיכוי)</t>
+          <t>מקורון פטיסרי (זיכוי בבנק)</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1210,24 +1210,24 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>חשבונית הכנסה להעברה</t>
+          <t>לא נמצא במייל מסמך על התנועה. לא ברור אם זה תשלום מלקוח או זיכוי. סכום זהה לחשבונית 20022 של עזריאלי</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>להוציא חשבונית הכנסה</t>
+          <t>לברר מול נעם ולהוציא חשבונית הכנסה</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>ד. הכנסות (מהקובץ, לא נחקר בחיפוש)</t>
+          <t>ד. הכנסות</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>לקוח: ג'ויה אור</t>
+          <t>ג'ויה (הפקדת שיק)</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1240,7 +1240,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>חשבונית הכנסה להפקדת שיק (פנינה חזרה על כך ב-18/10)</t>
+          <t>לא נמצאה חשבונית הכנסה (פנינה חזרה על כך ב-18/10)</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1252,17 +1252,17 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>ד. הכנסות (מהקובץ, לא נחקר בחיפוש)</t>
+          <t>ד. הכנסות</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>לקוח: ננוס לאנצ'</t>
+          <t>ננוס לאנצ'</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>02/03/26</t>
+          <t>מ-02/03/26</t>
         </is>
       </c>
       <c r="D27" s="2" t="n">
@@ -1270,68 +1270,130 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>5 חשבוניות מול 4 העברות. שיק 21078 לא הופקד (פנינה, 18/10)</t>
+          <t>ב-29/09 פנינה כתבה שיש 5 חשבוניות פתוחות מול 4 העברות: 20048, 20056, 20051, 20061, 20057, וזיכוי 1005 על חשבונית 20047. נשלחה לה כרטסת. שיק 21078 לא הופקד (18/10)</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>לבדוק איזו חשבונית פתוחה, ולהחליט מה לעשות עם השיק</t>
+          <t>להחליט איזו חשבונית נשארת פתוחה ולהפקיד את שיק 21078</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>ד. הכנסות (מהקובץ, לא נחקר בחיפוש)</t>
+          <t>ד. הכנסות</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>לקוחות עם יתרה פתוחה</t>
+          <t>ביט.ברידג (מלון קמפינסקי)</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>שונים</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="n"/>
+          <t>04/11/25</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>11800</v>
+      </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>מ.ד.ע עזריאלי: חשבונית 20022 (17,700 ₪), שולמו 8,850 ₪ ונשארו 8,850 ₪. ביט.ברידג (קמפינסקי): חשבונית 20044 (11,800 ₪). פיצריה בר דיזנגוף: חשבונית 40150 (9,440 ₪)</t>
+          <t>חשבונית 20044 על התשלום הראשון, לא שולמה. ב-28/12/25 נשלח ליעל מקמפינסקי חשבון עסקה 1024 על כל העסקה. ב-04/01/26 היא שאלה אם הופקה חשבונית עבורו. ב-03/03/26 נעם העביר הזמנת רכש PO26001309 וביקש חשבונית מס</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>לברר מול הלקוחות איך ייסגרו היתרות (בהערות בקובץ כתוב 'יודעת')</t>
+          <t>לברר מול קמפינסקי אם 20044 שולמה או הוחלפה בהזמנת הרכש</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
+          <t>ד. הכנסות</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>מ.ד.ע עזריאלי</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>29/07/26</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>8850</v>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>חשבונית 20022 על 17,700 ₪, שולמו 8,850 ₪ ב-29/07. נשארו 8,850 ₪ (במרץ נשלחה בקשת מקדמה של חצי)</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>לבדוק מתי ישולם היתרה</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>ד. הכנסות</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>פיצריה בר כיכר דיזנגוף</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>20/09/26</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>9440</v>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>חשבונית 40150, לא שולמה. חשבונית 40149 בוטלה כי התקבל ח.פ שגוי (05/10)</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>לוודא שהחשבונית שוחררה בח.פ הנכון, ולגבות</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
           <t>ה. תיקוני רשימה</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>רשימת התנועות הפתוחות</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>12/10/26</t>
         </is>
       </c>
-      <c r="D29" s="2" t="n">
+      <c r="D31" s="2" t="n">
         <v>453</v>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>בקובץ רשום 296 ₪ להעברה מ-12/10 לקבוצת העתקות. בבנק ובקבלה 244052 הסכום הוא 453 ₪</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>לתקן ברשימה לפני שליחה לפנינה</t>
         </is>

</xml_diff>

<commit_message>
Add Hatacot payment-to-receipt matching sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vhYGPaAM74nnJetAhxgmr
</commit_message>
<xml_diff>
--- a/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
+++ b/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="רשימת חסרים" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="תוצאות חיפוש" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מה חסר ממי לבקש" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="קבוצת העתקות - שיוך" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="תוצאות חיפוש" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מה חסר ממי לבקש" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1410,6 +1411,288 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="80" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>תאריך בבנק</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>סכום בבנק ₪</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>קבלה שסוגרת</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>תאריך הקבלה</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>חשבונית</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>הערה</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>17/06/26</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>385</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>240616</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>24/06/26</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>לא מצוין בקבלה</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>שתי העברות זהות באותו יום</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>17/06/26</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>385</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>240617</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>24/06/26</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>לא מצוין בקבלה</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>שתי העברות זהות באותו יום. החשבונית הקיימת (648740) על 296 ₪ בלבד, ולכן יתרת זכות של כ-474 ₪</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>לא בבנק</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>296</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>אין קבלה נפרדת</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>24/06/26</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>חשבונית מס 648740 על 296 ₪</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>שולמה מיתרת הזכות מההעברה של 385 ₪, לכן אין בבנק תשלום בסכום הזה</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>15/07/26</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>375</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>241875</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>05/08/26</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>650922 (375 ₪)</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>תואם</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>06/08/26</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>375</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>242606</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>27/08/26</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>650922 (כבר שולמה בקבלה 241875)</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>תשלום כפול אפשרי, יתרת זכות 375 ₪</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>10/09/26</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>453</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>243829</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>06/10/26</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>655014 (453 ₪)</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>תואם</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>12/10/26</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>453</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>244052</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>14/10/26</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>655014 (כבר שולמה ב-10/09)</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>תשלום כפול. בקבלה כתוב 'כפילות, ביתרת זכות'. ברשימת התנועות הפתוחות היה רשום 296 ₪, והסכום הנכון בבנק הוא 453 ₪</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>סיכום</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>יתרות זכות צפויות: 474 + 375 + 453 = כ-1,302 ₪. לאמת מול כרטסת לקוח של קבוצת העתקות</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2264,7 +2547,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Hatacot: confirm via customer ledger, credit balance 1,302
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vhYGPaAM74nnJetAhxgmr
</commit_message>
<xml_diff>
--- a/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
+++ b/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
@@ -1053,7 +1053,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>12/10, 06/08, 17/06</t>
+          <t>17/06, 06/08, 12/10</t>
         </is>
       </c>
       <c r="D20" s="2" t="n">
@@ -1061,12 +1061,12 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>יתרות זכות: 453 ₪ (תשלום כפול על 655014), 375 ₪ (תשלום כפול על 650922), כ-474 ₪ מיוני. סה"כ כ-1,300 ₪</t>
+          <t>יתרת זכות של 1,302 ₪ לפי כרטסת הלקוח מ-21/10/26: 89 מיוני, 385 (כפילות 240617), 375 (כפילות 242606) ו-453 (כפילות 244052)</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>חן וקנין: כרטסת, וקיזוז או החזר (הטיוטה במייל המשרד)</t>
+          <t>לבקש מקבוצת העתקות קיזוז מחשבוניות עתידיות או החזר</t>
         </is>
       </c>
     </row>
@@ -1475,12 +1475,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>לא מצוין בקבלה</t>
+          <t>648740 (296 ₪)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>שתי העברות זהות באותו יום</t>
+          <t>סוגרת את החשבונית. נשארו 89 ₪ יתרת זכות</t>
         </is>
       </c>
     </row>
@@ -1505,12 +1505,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>לא מצוין בקבלה</t>
+          <t>אין. רשומה בכרטסת כ"כפילות"</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>שתי העברות זהות באותו יום. החשבונית הקיימת (648740) על 296 ₪ בלבד, ולכן יתרת זכות של כ-474 ₪</t>
+          <t>תשלום כפול, יתרת זכות 385 ₪</t>
         </is>
       </c>
     </row>
@@ -1527,7 +1527,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>אין קבלה נפרדת</t>
+          <t>240616</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>שולמה מיתרת הזכות מההעברה של 385 ₪, לכן אין בבנק תשלום בסכום הזה</t>
+          <t>שולמה בקבלה 240616 (בהעברה של 385 ₪), לכן אין בבנק תשלום בסכום הזה</t>
         </is>
       </c>
     </row>
@@ -1678,7 +1678,7 @@
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>יתרות זכות צפויות: 474 + 375 + 453 = כ-1,302 ₪. לאמת מול כרטסת לקוח של קבוצת העתקות</t>
+          <t>יתרת זכות אצל קבוצת העתקות לפי הכרטסת מ-21/10/26: 1,302 ₪ (89 + 385 + 375 + 453). חיובים 1,124 ₪, זכויות 2,426 ₪. חשבונית 650922 הופקה ב-31/07/26 וחשבונית 655014 ב-30/09/26</t>
         </is>
       </c>
     </row>
@@ -1898,12 +1898,12 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>נמצא (שתי ההעברות, הקבלות הועלו לשיחה)</t>
+          <t>נמצא (נסגר, מאומת בכרטסת)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>קבלות 240616 ו-240617, שתיהן מ-24/06/26: כל אחת 385 ₪, העברה בנקאית מ-17/06/26. בכך שתי ההעברות מכוסות. ב-21/06 חן וקנין כתבה שחשבונית 648740 היא על 296 ₪ ושההעברה (385 ₪) עודפת, והשאירה כיתרת זכות. כיוון ששולמו 770 ₪ על חשבונית של 296 ₪, נשארה אצלם יתרת זכות של כ-474 ₪. לא ברור אם היא משקפת תשלום כפול או תשלום מראש, וכדאי לאמת מולם.</t>
+          <t>לפי כרטסת הלקוח של קבוצת העתקות (הופקה ב-21/10/26): קבלה 240616 (385 ₪, העברה מ-17/06) סוגרת את חשבונית 648740 על 296 ₪, וקבלה 240617 (385 ₪, העברה מ-17/06) רשומה בכרטסת כ"כפילות". כלומר ההעברה השנייה של 385 ₪ היא תשלום כפול, ובנוסף נשארו 89 ₪ יתרה מהראשונה.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Eshkol 4U: details from invoice IN264000182
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vhYGPaAM74nnJetAhxgmr
</commit_message>
<xml_diff>
--- a/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
+++ b/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
@@ -1091,12 +1091,12 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>חשבוניות 18 (70.91 ₪) ו-182 (86 ₪): לא נמצא חיוב בבנק</t>
+          <t>חשבונית IN264000182 מ-28/02/26: 86 ₪ (72.88 + מע"מ 13.12), עבור שירותי תפעול (פעולת חוק מינימלי 02/26), לתשלום עד 31/03/26 בהעברה בנקאית לבנק לאומי (10) סניף 800 חשבון 520258/04. לא נמצא חיוב. את חשבונית 18 (70.91 ₪, ינואר) לא מצאתי בדרייב. בתיבה יש מיילים חודשיים מקבוצת שקל (sharonfi@shekelgroup.co.il) מ-11/01 ומ-17/03/26 עם פירוט חיוב לשירותי תפעול, בקישור מוגן בסיסמה ב-SMS</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>לבדוק באשראי / לשאול את אשכול 4U איך שולם</t>
+          <t>לבדוק בבנק העברה ללאומי 800/520258 בסביבות 31/03 ו-ינואר-פברואר, או לבקש מקבוצת שקל (sharonfi@shekelgroup.co.il) איך החיוב נגבה</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Galaxy: credit balance per Margalit
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vhYGPaAM74nnJetAhxgmr
</commit_message>
<xml_diff>
--- a/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
+++ b/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
@@ -1121,12 +1121,12 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>חשבונית 723 על 503 ₪ מול העברה של 475 ₪: חסרים 28 ₪</t>
+          <t>חשבונית 723 על 503 ₪ מול העברה של 475 ₪. ברשימת פנינה נכתב שחייבים להם 28 ₪, אבל לפי מרגלית יש לחברה יתרת זכות אצל גלקסי, כלומר אין חוב. הנתון לא אומת מול כרטסת</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>לסגור מול גלקסי</t>
+          <t>לתקן את ההערה ברשימה של פנינה, ולהשתמש ביתרת הזכות בחשבון הבא</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tirosh invoice 114720 found in Drive
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vhYGPaAM74nnJetAhxgmr
</commit_message>
<xml_diff>
--- a/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
+++ b/output/חשבוניות_חסרות_תוצאות_חיפוש_מייל_המשרד.xlsx
@@ -775,7 +775,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>א. הוצאות: חשבונית לא נמצאה</t>
+          <t>ב. נמצא, ממתין לשליחה לביזיבוקס</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -793,12 +793,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>חשבונית מס סופית (המתוקנת מ-keren.m@tiroche.co.il לא נמצאת בתיבת המשרד, צריך לוודא שאינה טיוטה)</t>
+          <t>חשבונית מס/קבלה 114720 נמצאה בדרייב, בתיקיית "להעביר לפנינה". כדאי לוודא שהיא חתומה</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>נועם / keren.m@tiroche.co.il</t>
+          <t>לוודא מול הגלריה ולשלוח לביזיבוקס או לפנינה</t>
         </is>
       </c>
     </row>
@@ -2514,7 +2514,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>אוראגן תירוש (לבדוק)</t>
+          <t>אוראגן תירוש</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -2525,20 +2525,24 @@
       <c r="C25" s="2" t="n">
         <v>8322</v>
       </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>לא נמצא</t>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>נמצא (בדרייב, בתיקיית "להעביר לפנינה")</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>חיפוש 'תירוש' / 'tiroche' לא החזיר מייל בתיבת המשרד. החשבונית המתוקנת מ-keren.m@tiroche.co.il לא נמצאת כאן, ולכן אי אפשר לאמת אם היא סופית או טיוטה.</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr"/>
+          <t>קובץ "2026-03-20 חשבונית 114720 - קדישמן כבשים - 8,322 ש"ח.pdf" בדרייב של המשרד, תיקיית "להעביר לפנינה". חשבונית מס/קבלה 114720 מ-20/03/26 של אוראגן תירוש בע"מ: 6,864 ₪ + עמלה 1,236 + מע"מ 18% (222) = 8,322 ₪, עבור רכישת ציור (מנשה קדישמן, "כבשים"), שולם בהעברה. הקובץ הוא הדפסה לקובץ PDF ממערכת הגלריה ועם סימן "TRIAL MODE" של תוכנת ההדפסה, ולא חשבונית דיגיטלית חתומה, ולכן כדאי לוודא מול הגלריה (keren.m@tiroche.co.il) אם יש גרסה חתומה</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>קובץ בדרייב: https://drive.google.com/file/d/17Aowl9qEFIOOjfQQqB-STzWtjLBXGaTf/view</t>
+        </is>
+      </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>לא ידוע</t>
+          <t>לא ידוע (בתיקיית "להעביר לפנינה")</t>
         </is>
       </c>
     </row>

</xml_diff>